<commit_message>
Use static relative hyperlinks for BSI.IT.6.C7.3 evidence links
The =HYPERLINK(EvidenceRoot&...) formulas depended on CELL("filename") and
recalculation, so they did not open in Protected View, from inside a zip or
in Excel Online. All 278 evidence file and folder links are now plain
hyperlinks relative to the workbook's folder (BSI.IT.6.C7.3-Evidences\...).
WP Summary link-setting notes updated (Hyperlink base for other locations).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZXJw9RbzX4wjsjHgupSGR
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence.xlsx
@@ -31,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="40">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -246,6 +246,19 @@
     </font>
     <font>
       <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
       <u val="single"/>
     </font>
   </fonts>
@@ -475,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -659,6 +672,13 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2052,6 +2072,7 @@
     <row r="22" ht="27.2" customHeight="1"/>
     <row r="23" ht="20.45" customHeight="1"/>
     <row r="24" ht="20.45" customHeight="1"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="71" t="inlineStr">
         <is>
@@ -2071,7 +2092,7 @@
       <c r="E27" s="74" t="n"/>
       <c r="F27" s="63" t="inlineStr">
         <is>
-          <t>Yellow cell: leave blank if the evidence folder sits next to this workbook; otherwise paste its full path (local, network or SharePoint).</t>
+          <t>Links are relative to this workbook: keep the folder BSI.IT.6.C7.3-Evidences next to this .xlsx (extract the whole zip first; do not open the workbook from inside the zip). If the evidence sits elsewhere, set File &gt; Info &gt; Properties &gt; Advanced Properties &gt; Summary &gt; Hyperlink base to the folder that contains it.</t>
         </is>
       </c>
     </row>
@@ -2081,18 +2102,21 @@
           <t>Links resolve to</t>
         </is>
       </c>
-      <c r="B28" s="75">
-        <f>EvidenceRoot</f>
-        <v/>
+      <c r="B28" s="75" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\ (in the same folder as this workbook)</t>
+        </is>
       </c>
       <c r="C28" s="73" t="n"/>
       <c r="D28" s="73" t="n"/>
       <c r="E28" s="74" t="n"/>
-      <c r="F28" s="76">
-        <f>HYPERLINK(EvidenceRoot,"Test: open the evidence folder")</f>
-        <v/>
-      </c>
-    </row>
+      <c r="F28" s="82" t="inlineStr">
+        <is>
+          <t>Test: open the evidence folder</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="71" t="inlineStr">
         <is>
@@ -2106,9 +2130,10 @@
           <t>Folder 01</t>
         </is>
       </c>
-      <c r="B31" s="79">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications")</f>
-        <v/>
+      <c r="B31" s="79" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications</t>
+        </is>
       </c>
       <c r="C31" s="73" t="n"/>
       <c r="D31" s="73" t="n"/>
@@ -2125,9 +2150,10 @@
           <t>Folder 02</t>
         </is>
       </c>
-      <c r="B32" s="79">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B32" s="79" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="C32" s="73" t="n"/>
       <c r="D32" s="73" t="n"/>
@@ -2144,9 +2170,10 @@
           <t>Folder 03</t>
         </is>
       </c>
-      <c r="B33" s="79">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B33" s="79" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="C33" s="73" t="n"/>
       <c r="D33" s="73" t="n"/>
@@ -2163,9 +2190,10 @@
           <t>Folder 04</t>
         </is>
       </c>
-      <c r="B34" s="79">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B34" s="79" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="C34" s="73" t="n"/>
       <c r="D34" s="73" t="n"/>
@@ -2182,9 +2210,10 @@
           <t>Folder 05</t>
         </is>
       </c>
-      <c r="B35" s="79">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails")</f>
-        <v/>
+      <c r="B35" s="79" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails</t>
+        </is>
       </c>
       <c r="C35" s="73" t="n"/>
       <c r="D35" s="73" t="n"/>
@@ -2218,6 +2247,14 @@
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B28:E28"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" display="Test: open the evidence folder" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos"&amp;1 &amp;K000000 Confidential#_x000d_</oddHeader>
@@ -4513,6 +4550,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4" ht="21.95" customHeight="1">
       <c r="A4" s="46" t="inlineStr">
         <is>
@@ -4985,6 +5023,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="64" t="inlineStr">
         <is>
@@ -5006,6 +5045,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="64" t="inlineStr">
         <is>
@@ -5035,9 +5075,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="80">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open evidence folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="A22" s="80" t="inlineStr">
+        <is>
+          <t>Open evidence folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5047,6 +5088,9 @@
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A19:H19"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" display="Open evidence folder 05: DRS01, DRS02" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos"&amp;1 &amp;K000000 Confidential#_x000d_</oddHeader>
@@ -5057,7 +5101,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5445,25 +5489,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T3" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U3" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA01")</f>
-        <v/>
-      </c>
-      <c r="V3" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA01, DMA02")</f>
-        <v/>
-      </c>
-      <c r="W3" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E09, E16b")</f>
-        <v/>
-      </c>
-      <c r="X3" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T3" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U3" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA01</t>
+        </is>
+      </c>
+      <c r="V3" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA01, DMA02</t>
+        </is>
+      </c>
+      <c r="W3" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E09, E16b</t>
+        </is>
+      </c>
+      <c r="X3" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -5584,25 +5633,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T4" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U4" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA01")</f>
-        <v/>
-      </c>
-      <c r="V4" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA01, DMA02")</f>
-        <v/>
-      </c>
-      <c r="W4" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E09, E16b")</f>
-        <v/>
-      </c>
-      <c r="X4" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T4" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U4" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA01</t>
+        </is>
+      </c>
+      <c r="V4" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA01, DMA02</t>
+        </is>
+      </c>
+      <c r="W4" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E09, E16b</t>
+        </is>
+      </c>
+      <c r="X4" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -5723,25 +5777,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Claudia Romero). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T5" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U5" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA01")</f>
-        <v/>
-      </c>
-      <c r="V5" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA01, DMA02")</f>
-        <v/>
-      </c>
-      <c r="W5" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E09, E16b")</f>
-        <v/>
-      </c>
-      <c r="X5" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T5" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U5" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA01</t>
+        </is>
+      </c>
+      <c r="V5" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA01, DMA02</t>
+        </is>
+      </c>
+      <c r="W5" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E09, E16b</t>
+        </is>
+      </c>
+      <c r="X5" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -5884,25 +5943,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Claudia Romero, Miguel Orozco, Maria del Cerro Hontanilla). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T6" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U6" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA01, BLA02")</f>
-        <v/>
-      </c>
-      <c r="V6" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA01, DMA02, DMA05, DMA11")</f>
-        <v/>
-      </c>
-      <c r="W6" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E09, E16b")</f>
-        <v/>
-      </c>
-      <c r="X6" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T6" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U6" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA01, BLA02</t>
+        </is>
+      </c>
+      <c r="V6" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA01, DMA02, DMA05, DMA11</t>
+        </is>
+      </c>
+      <c r="W6" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E09, E16b</t>
+        </is>
+      </c>
+      <c r="X6" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6022,25 +6086,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Michelle Oropesa). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T7" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U7" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA04")</f>
-        <v/>
-      </c>
-      <c r="V7" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA02, DMA04")</f>
-        <v/>
-      </c>
-      <c r="W7" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E16b")</f>
-        <v/>
-      </c>
-      <c r="X7" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T7" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U7" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA04</t>
+        </is>
+      </c>
+      <c r="V7" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA02, DMA04</t>
+        </is>
+      </c>
+      <c r="W7" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E16b</t>
+        </is>
+      </c>
+      <c r="X7" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6163,25 +6232,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Franklin Puentes). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T8" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U8" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA03")</f>
-        <v/>
-      </c>
-      <c r="V8" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA02, DMA03")</f>
-        <v/>
-      </c>
-      <c r="W8" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b")</f>
-        <v/>
-      </c>
-      <c r="X8" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T8" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U8" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA03</t>
+        </is>
+      </c>
+      <c r="V8" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA02, DMA03</t>
+        </is>
+      </c>
+      <c r="W8" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b</t>
+        </is>
+      </c>
+      <c r="X8" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6317,25 +6391,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Franklin Puentes, Maria del Cerro Hontanilla). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T9" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U9" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA02, BLA03")</f>
-        <v/>
-      </c>
-      <c r="V9" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA02, DMA03, DMA05")</f>
-        <v/>
-      </c>
-      <c r="W9" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b")</f>
-        <v/>
-      </c>
-      <c r="X9" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T9" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U9" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA02, BLA03</t>
+        </is>
+      </c>
+      <c r="V9" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA02, DMA03, DMA05</t>
+        </is>
+      </c>
+      <c r="W9" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b</t>
+        </is>
+      </c>
+      <c r="X9" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6456,25 +6535,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Sadis Alvarenga Hernandez). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T10" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U10" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA05, BLA06")</f>
-        <v/>
-      </c>
-      <c r="V10" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA02")</f>
-        <v/>
-      </c>
-      <c r="W10" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E10, E16b")</f>
-        <v/>
-      </c>
-      <c r="X10" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T10" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U10" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA05, BLA06</t>
+        </is>
+      </c>
+      <c r="V10" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA02</t>
+        </is>
+      </c>
+      <c r="W10" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E10, E16b</t>
+        </is>
+      </c>
+      <c r="X10" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6602,25 +6686,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (David Marquez, Michelle Oropesa). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T11" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U11" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA03, BLA04")</f>
-        <v/>
-      </c>
-      <c r="V11" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA02, DMA04")</f>
-        <v/>
-      </c>
-      <c r="W11" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b")</f>
-        <v/>
-      </c>
-      <c r="X11" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T11" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U11" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA03, BLA04</t>
+        </is>
+      </c>
+      <c r="V11" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA02, DMA04</t>
+        </is>
+      </c>
+      <c r="W11" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b</t>
+        </is>
+      </c>
+      <c r="X11" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="60.6" customFormat="1" customHeight="1" s="8">
@@ -6818,25 +6907,30 @@
           <t>PASS. DIV executed and validated during the 11/15/2025 annual DR exercise, application in scope (MA01), results documented in BCiC/BCMS and approved by business line management (Ricardo Garcia, David Marquez, Claudia Romero, Miguel Orozco, Sadis Alvarenga Hernandez, Maria del Cerro Hontanilla, Michelle Oropesa, Franklin Puentes, Martha Sullivan, Liliana Vizhnay, Victoria Fernandez, Xavier Caisapanta, Clara De Castro). IT and business DR scope confirmed by the DRS01 (IT Scope) and DRS02 (Business Scope) emails.</t>
         </is>
       </c>
-      <c r="T12" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"Open folder 01: MA01")</f>
-        <v/>
-      </c>
-      <c r="U12" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"Open folder 02: BLA01, BLA02, BLA03, BLA04, BLA05, BLA06")</f>
-        <v/>
-      </c>
-      <c r="V12" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"Open folder 03: DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12")</f>
-        <v/>
-      </c>
-      <c r="W12" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"Open folder 04: E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b")</f>
-        <v/>
-      </c>
-      <c r="X12" s="81">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"Open folder 05: DRS01, DRS02")</f>
-        <v/>
+      <c r="T12" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 01: MA01</t>
+        </is>
+      </c>
+      <c r="U12" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 02: BLA01, BLA02, BLA03, BLA04, BLA05, BLA06</t>
+        </is>
+      </c>
+      <c r="V12" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 03: DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12</t>
+        </is>
+      </c>
+      <c r="W12" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 04: E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b</t>
+        </is>
+      </c>
+      <c r="X12" s="81" t="inlineStr">
+        <is>
+          <t>Open folder 05: DRS01, DRS02</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="60.6" customHeight="1">
@@ -6881,28 +6975,78 @@
     <hyperlink ref="S2" location="'Application Attribute Testing'!A113" tooltip="Go to conclusion table" display="Control Sample Assessment Result (Pass/Fail)"/>
     <hyperlink ref="A3" location="'Application Attribute Testing'!A115" tooltip="Go to sample 1822 conclusion" display="'Application Attribute Testing'!A115"/>
     <hyperlink ref="R3" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA01: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" display="Open folder 01: MA01" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" display="Open folder 02: BLA01" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" display="Open folder 03: DMA01, DMA02" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" display="Open folder 04: E01, E02, E03, E04, E05, E09, E16b" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" display="Open folder 05: DRS01, DRS02" r:id="rId5"/>
     <hyperlink ref="A4" location="'Application Attribute Testing'!A116" tooltip="Go to sample 1867 conclusion" display="'Application Attribute Testing'!A116"/>
     <hyperlink ref="R4" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA01: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" display="Open folder 01: MA01" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" display="Open folder 02: BLA01" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" display="Open folder 03: DMA01, DMA02" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" display="Open folder 04: E01, E02, E03, E04, E05, E09, E16b" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" display="Open folder 05: DRS01, DRS02" r:id="rId10"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A117" tooltip="Go to sample 1868 conclusion" display="'Application Attribute Testing'!A117"/>
     <hyperlink ref="R5" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA01: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" display="Open folder 01: MA01" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" display="Open folder 02: BLA01" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V5" display="Open folder 03: DMA01, DMA02" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" display="Open folder 04: E01, E02, E03, E04, E05, E09, E16b" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" display="Open folder 05: DRS01, DRS02" r:id="rId15"/>
     <hyperlink ref="A6" location="'Application Attribute Testing'!A118" tooltip="Go to sample 3299 conclusion" display="'Application Attribute Testing'!A118"/>
     <hyperlink ref="R6" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA01: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" display="Open folder 01: MA01" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" display="Open folder 02: BLA01, BLA02" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V6" display="Open folder 03: DMA01, DMA02, DMA05, DMA11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" display="Open folder 04: E01, E02, E03, E04, E05, E09, E16b" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" display="Open folder 05: DRS01, DRS02" r:id="rId20"/>
     <hyperlink ref="A7" location="'Application Attribute Testing'!A119" tooltip="Go to sample 4052 conclusion" display="'Application Attribute Testing'!A119"/>
     <hyperlink ref="R7" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA04: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" display="Open folder 01: MA01" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" display="Open folder 02: BLA04" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" display="Open folder 03: DMA02, DMA04" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" display="Open folder 04: E01, E02, E03, E04, E05, E16b" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" display="Open folder 05: DRS01, DRS02" r:id="rId25"/>
     <hyperlink ref="A8" location="'Application Attribute Testing'!A120" tooltip="Go to sample 3301 conclusion" display="'Application Attribute Testing'!A120"/>
     <hyperlink ref="R8" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA03: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" display="Open folder 01: MA01" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" display="Open folder 02: BLA03" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V8" display="Open folder 03: DMA02, DMA03" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" display="Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" display="Open folder 05: DRS01, DRS02" r:id="rId30"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A121" tooltip="Go to sample 1903 conclusion" display="'Application Attribute Testing'!A121"/>
     <hyperlink ref="R9" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA02: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" display="Open folder 01: MA01" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" display="Open folder 02: BLA02, BLA03" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" display="Open folder 03: DMA02, DMA03, DMA05" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" display="Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" display="Open folder 05: DRS01, DRS02" r:id="rId35"/>
     <hyperlink ref="A10" location="'Application Attribute Testing'!A122" tooltip="Go to sample 1917 conclusion" display="'Application Attribute Testing'!A122"/>
     <hyperlink ref="R10" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA05: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" display="Open folder 01: MA01" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" display="Open folder 02: BLA05, BLA06" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" display="Open folder 03: DMA02" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" display="Open folder 04: E01, E02, E03, E04, E05, E10, E16b" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" display="Open folder 05: DRS01, DRS02" r:id="rId40"/>
     <hyperlink ref="A11" location="'Application Attribute Testing'!A123" tooltip="Go to sample 1936 conclusion" display="'Application Attribute Testing'!A123"/>
     <hyperlink ref="R11" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA03: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T11" display="Open folder 01: MA01" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" display="Open folder 02: BLA03, BLA04" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" display="Open folder 03: DMA02, DMA04" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" display="Open folder 04: E01, E02, E03, E04, E05, E07, E08, E16b" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" display="Open folder 05: DRS01, DRS02" r:id="rId45"/>
     <hyperlink ref="A12" location="'Application Attribute Testing'!A124" tooltip="Go to sample 1937 conclusion" display="'Application Attribute Testing'!A124"/>
     <hyperlink ref="R12" location="'Application Attribute Testing'!A71" tooltip="Go to evidence file reviews" display="[01 Management Attestation / In-Scope Applications]_x000a_MA01: BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png_x000a_[02 Business Line Approval Results: Email]_x000a_BLA01: BSI.IT.6.C7.3-Evidences\02_Business"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" display="Open folder 01: MA01" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" display="Open folder 02: BLA01, BLA02, BLA03, BLA04, BLA05, BLA06" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" display="Open folder 03: DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" display="Open folder 04: E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" display="Open folder 05: DRS01, DRS02" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7026,9 +7170,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B5" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
         <is>
@@ -7183,9 +7328,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B9" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B9" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
@@ -7340,9 +7486,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B13" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B13" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
@@ -7492,9 +7639,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B17" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B17" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
@@ -7644,9 +7792,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B21" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B21" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
@@ -7795,9 +7944,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B25" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B25" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
@@ -7947,9 +8097,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B29" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B29" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
@@ -8104,9 +8255,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B33" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B33" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
@@ -8261,9 +8413,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B37" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B37" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
@@ -8410,9 +8563,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B41" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B41" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C41" s="33" t="inlineStr">
         <is>
@@ -8468,9 +8622,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B42" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B42" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
@@ -8515,9 +8670,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B43" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B43" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C43" s="33" t="inlineStr">
         <is>
@@ -8561,9 +8717,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B44" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B44" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C44" s="33" t="inlineStr">
         <is>
@@ -8606,9 +8763,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B45" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B45" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C45" s="33" t="inlineStr">
         <is>
@@ -8741,9 +8899,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B49" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B49" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C49" s="33" t="inlineStr">
         <is>
@@ -8889,9 +9048,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B53" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B53" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C53" s="33" t="inlineStr">
         <is>
@@ -9040,9 +9200,10 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B57" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
+      <c r="B57" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
       </c>
       <c r="C57" s="33" t="inlineStr">
         <is>
@@ -9193,9 +9354,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B61" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B61" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C61" s="33" t="inlineStr">
         <is>
@@ -9252,9 +9414,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B62" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B62" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C62" s="33" t="inlineStr">
         <is>
@@ -9299,9 +9462,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B63" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B63" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C63" s="33" t="inlineStr">
         <is>
@@ -9345,9 +9509,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B64" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B64" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C64" s="33" t="inlineStr">
         <is>
@@ -9390,9 +9555,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B65" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B65" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C65" s="33" t="inlineStr">
         <is>
@@ -9525,9 +9691,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B69" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B69" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C69" s="33" t="inlineStr">
         <is>
@@ -9657,9 +9824,10 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B73" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B73" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C73" s="33" t="inlineStr">
         <is>
@@ -9698,9 +9866,10 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B74" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B74" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C74" s="33" t="inlineStr">
         <is>
@@ -9739,9 +9908,10 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B75" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B75" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C75" s="33" t="inlineStr">
         <is>
@@ -9780,9 +9950,10 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B76" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
-        <v/>
+      <c r="B76" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
+        </is>
       </c>
       <c r="C76" s="33" t="inlineStr">
         <is>
@@ -9821,9 +9992,10 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B77" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B77" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C77" s="33" t="inlineStr">
         <is>
@@ -9862,9 +10034,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B78" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B78" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C78" s="33" t="inlineStr">
         <is>
@@ -9972,9 +10145,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B82" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B82" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C82" s="33" t="inlineStr">
         <is>
@@ -10008,9 +10182,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B83" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B83" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C83" s="33" t="inlineStr">
         <is>
@@ -10044,9 +10219,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B84" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B84" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C84" s="33" t="inlineStr">
         <is>
@@ -10080,9 +10256,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B85" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B85" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C85" s="33" t="inlineStr">
         <is>
@@ -10116,9 +10293,10 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B86" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
-        <v/>
+      <c r="B86" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C86" s="33" t="inlineStr">
         <is>
@@ -10152,9 +10330,10 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B87" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
-        <v/>
+      <c r="B87" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C87" s="33" t="inlineStr">
         <is>
@@ -10188,9 +10367,10 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B88" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
-        <v/>
+      <c r="B88" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C88" s="33" t="inlineStr">
         <is>
@@ -10224,9 +10404,10 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B89" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
-        <v/>
+      <c r="B89" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C89" s="33" t="inlineStr">
         <is>
@@ -10260,9 +10441,10 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B90" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
-        <v/>
+      <c r="B90" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C90" s="33" t="inlineStr">
         <is>
@@ -10296,9 +10478,10 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B91" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
-        <v/>
+      <c r="B91" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
+        </is>
       </c>
       <c r="C91" s="33" t="inlineStr">
         <is>
@@ -10332,9 +10515,10 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B92" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
-        <v/>
+      <c r="B92" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C92" s="33" t="inlineStr">
         <is>
@@ -10368,9 +10552,10 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B93" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
-        <v/>
+      <c r="B93" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C93" s="33" t="inlineStr">
         <is>
@@ -10404,9 +10589,10 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B94" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
-        <v/>
+      <c r="B94" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
+        </is>
       </c>
       <c r="C94" s="33" t="inlineStr">
         <is>
@@ -10499,9 +10685,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B98" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B98" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C98" s="33" t="inlineStr">
         <is>
@@ -10535,9 +10722,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B99" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B99" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C99" s="33" t="inlineStr">
         <is>
@@ -10571,9 +10759,10 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B100" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
-        <v/>
+      <c r="B100" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+        </is>
       </c>
       <c r="C100" s="33" t="inlineStr">
         <is>
@@ -10607,9 +10796,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B101" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B101" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C101" s="33" t="inlineStr">
         <is>
@@ -10643,9 +10833,10 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B102" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
-        <v/>
+      <c r="B102" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+        </is>
       </c>
       <c r="C102" s="33" t="inlineStr">
         <is>
@@ -10679,9 +10870,10 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B103" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
+      <c r="B103" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
       </c>
       <c r="C103" s="33" t="inlineStr">
         <is>
@@ -10715,9 +10907,10 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B104" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
-        <v/>
+      <c r="B104" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C104" s="33" t="inlineStr">
         <is>
@@ -10751,9 +10944,10 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B105" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
-        <v/>
+      <c r="B105" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C105" s="33" t="inlineStr">
         <is>
@@ -10787,9 +10981,10 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B106" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
-        <v/>
+      <c r="B106" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+        </is>
       </c>
       <c r="C106" s="33" t="inlineStr">
         <is>
@@ -10823,9 +11018,10 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B107" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
-        <v/>
+      <c r="B107" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+        </is>
       </c>
       <c r="C107" s="33" t="inlineStr">
         <is>
@@ -10859,9 +11055,10 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B108" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
-        <v/>
+      <c r="B108" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+        </is>
       </c>
       <c r="C108" s="33" t="inlineStr">
         <is>
@@ -10895,9 +11092,10 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B109" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
-        <v/>
+      <c r="B109" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
       </c>
       <c r="C109" s="33" t="inlineStr">
         <is>
@@ -11672,42 +11870,96 @@
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing-1'!B2" tooltip="Back to column B on Application Attribute Testing-1" display="1. Application Name (column B): review of evidence files and results"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A98" tooltip="Go to MA01 evidence review" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId1"/>
     <hyperlink ref="A7" location="'Application Attribute Testing-1'!C2" tooltip="Back to column C on Application Attribute Testing-1" display="2. Applications in Scope Identified (column C): review of evidence files and results"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A98" tooltip="Go to MA01 evidence review" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId2"/>
     <hyperlink ref="A11" location="'Application Attribute Testing-1'!D2" tooltip="Back to column D on Application Attribute Testing-1" display="3. IT DR exercise name (column D): review of evidence files and results"/>
     <hyperlink ref="A13" location="'Application Attribute Testing'!A99" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId3"/>
     <hyperlink ref="A15" location="'Application Attribute Testing-1'!E2" tooltip="Back to column E on Application Attribute Testing-1" display="4. IT DR exercise name, was the exercise annually executed? (column E): review of evidence files and results"/>
     <hyperlink ref="A17" location="'Application Attribute Testing'!A99" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId4"/>
     <hyperlink ref="A19" location="'Application Attribute Testing-1'!F2" tooltip="Back to column F on Application Attribute Testing-1" display="5. Business Tester (column F): review of evidence files and results"/>
     <hyperlink ref="A21" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId5"/>
     <hyperlink ref="A23" location="'Application Attribute Testing-1'!G2" tooltip="Back to column G on Application Attribute Testing-1" display="6. Business Data validation (column G): review of evidence files and results"/>
     <hyperlink ref="A25" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId6"/>
     <hyperlink ref="A27" location="'Application Attribute Testing-1'!H2" tooltip="Back to column H on Application Attribute Testing-1" display="7. Business line manager name (column H): review of evidence files and results"/>
     <hyperlink ref="A29" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId7"/>
     <hyperlink ref="A31" location="'Application Attribute Testing-1'!I2" tooltip="Back to column I on Application Attribute Testing-1" display="8. Business line manager approval dates (column I): review of evidence files and results"/>
     <hyperlink ref="A33" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId8"/>
     <hyperlink ref="A35" location="'Application Attribute Testing-1'!J2" tooltip="Back to column J on Application Attribute Testing-1" display="9. DIV Test procedures listed within the Test results document (column J): review of evidence files and results"/>
     <hyperlink ref="A37" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId9"/>
     <hyperlink ref="A39" location="'Application Attribute Testing-1'!K2" tooltip="Back to column K on Application Attribute Testing-1" display="10. Emails showing Business line manager approval of DIV testing results (column K): review of evidence files and results"/>
     <hyperlink ref="A41" location="'Application Attribute Testing'!A78" tooltip="Go to BLA06 evidence review" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId10"/>
     <hyperlink ref="A42" location="'Application Attribute Testing'!A82" tooltip="Go to DMA01 evidence review" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId11"/>
     <hyperlink ref="A43" location="'Application Attribute Testing'!A83" tooltip="Go to DMA02 evidence review" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId12"/>
     <hyperlink ref="A44" location="'Application Attribute Testing'!A84" tooltip="Go to DMA03 evidence review" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId13"/>
     <hyperlink ref="A45" location="'Application Attribute Testing'!A85" tooltip="Go to DMA04 evidence review" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId14"/>
     <hyperlink ref="A47" location="'Application Attribute Testing-1'!L2" tooltip="Back to column L on Application Attribute Testing-1" display="11. All evidence of Data Integrity DR test in BCIC (column L): review of evidence files and results"/>
     <hyperlink ref="A49" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId15"/>
     <hyperlink ref="A51" location="'Application Attribute Testing-1'!M2" tooltip="Back to column M on Application Attribute Testing-1" display="12. Annual Testing Executed (column M): review of evidence files and results"/>
     <hyperlink ref="A53" location="'Application Attribute Testing'!A99" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId16"/>
     <hyperlink ref="A55" location="'Application Attribute Testing-1'!N2" tooltip="Back to column N on Application Attribute Testing-1" display="13. Data Integrity Validation Performed by IT DR Team (column N): review of evidence files and results"/>
     <hyperlink ref="A57" location="'Application Attribute Testing'!A103" tooltip="Go to E05 evidence review" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId17"/>
     <hyperlink ref="A59" location="'Application Attribute Testing-1'!O2" tooltip="Back to column O on Application Attribute Testing-1" display="14. Business Line Approval of Results (column O): review of evidence files and results"/>
     <hyperlink ref="A61" location="'Application Attribute Testing'!A78" tooltip="Go to BLA06 evidence review" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId18"/>
     <hyperlink ref="A62" location="'Application Attribute Testing'!A82" tooltip="Go to DMA01 evidence review" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId19"/>
     <hyperlink ref="A63" location="'Application Attribute Testing'!A83" tooltip="Go to DMA02 evidence review" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId20"/>
     <hyperlink ref="A64" location="'Application Attribute Testing'!A84" tooltip="Go to DMA03 evidence review" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId21"/>
     <hyperlink ref="A65" location="'Application Attribute Testing'!A85" tooltip="Go to DMA04 evidence review" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId22"/>
     <hyperlink ref="A67" location="'Application Attribute Testing-1'!P2" tooltip="Back to column P on Application Attribute Testing-1" display="15. Results Documented in BCMS (column P): review of evidence files and results"/>
     <hyperlink ref="A69" location="'Application Attribute Testing'!A101" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx" r:id="rId54"/>
     <hyperlink ref="A115" location="'Application Attribute Testing-1'!A3" tooltip="Back to sample 1822 on Application Attribute Testing-1" display="1822"/>
     <hyperlink ref="B115" location="'Application Attribute Testing-1'!A3" tooltip="Back to sample 1822 on Application Attribute Testing-1" display="ACH Express"/>
     <hyperlink ref="A116" location="'Application Attribute Testing-1'!A4" tooltip="Back to sample 1867 on Application Attribute Testing-1" display="1867"/>
@@ -12011,9 +12263,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B5" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
         <is>
@@ -12314,9 +12567,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B9" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B9" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
@@ -12419,9 +12673,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B10" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B10" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
@@ -12471,9 +12726,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B11" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B11" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
@@ -12730,9 +12986,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B15" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B15" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
@@ -12827,9 +13084,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B16" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B16" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
@@ -12879,9 +13137,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B17" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B17" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
@@ -13129,9 +13388,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B21" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B21" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
@@ -13227,9 +13487,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B22" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B22" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -13279,9 +13540,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B23" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B23" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C23" s="33" t="inlineStr">
         <is>
@@ -13529,9 +13791,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B27" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B27" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
@@ -13823,9 +14086,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B31" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B31" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
@@ -14117,9 +14381,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B35" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B35" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
@@ -14213,9 +14478,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B36" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B36" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
@@ -14473,9 +14739,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B40" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B40" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C40" s="33" t="inlineStr">
         <is>
@@ -14767,9 +15034,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B44" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B44" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C44" s="33" t="inlineStr">
         <is>
@@ -15061,9 +15329,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B48" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B48" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C48" s="33" t="inlineStr">
         <is>
@@ -15149,9 +15418,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B49" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B49" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C49" s="33" t="inlineStr">
         <is>
@@ -15240,9 +15510,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B50" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B50" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C50" s="33" t="inlineStr">
         <is>
@@ -15330,9 +15601,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B51" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B51" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C51" s="33" t="inlineStr">
         <is>
@@ -15419,9 +15691,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B52" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B52" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C52" s="33" t="inlineStr">
         <is>
@@ -15706,9 +15979,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B56" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B56" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C56" s="33" t="inlineStr">
         <is>
@@ -16000,9 +16274,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B60" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B60" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C60" s="33" t="inlineStr">
         <is>
@@ -16098,9 +16373,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B61" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B61" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C61" s="33" t="inlineStr">
         <is>
@@ -16150,9 +16426,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B62" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B62" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C62" s="33" t="inlineStr">
         <is>
@@ -16400,9 +16677,10 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B66" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
+      <c r="B66" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
       </c>
       <c r="C66" s="33" t="inlineStr">
         <is>
@@ -16496,9 +16774,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B67" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B67" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C67" s="33" t="inlineStr">
         <is>
@@ -16548,9 +16827,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B68" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B68" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C68" s="33" t="inlineStr">
         <is>
@@ -16798,9 +17078,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B72" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B72" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C72" s="33" t="inlineStr">
         <is>
@@ -16886,9 +17167,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B73" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B73" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C73" s="33" t="inlineStr">
         <is>
@@ -16977,9 +17259,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B74" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B74" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C74" s="33" t="inlineStr">
         <is>
@@ -17067,9 +17350,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B75" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B75" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C75" s="33" t="inlineStr">
         <is>
@@ -17156,9 +17440,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B76" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B76" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C76" s="33" t="inlineStr">
         <is>
@@ -17245,9 +17530,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B77" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B77" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C77" s="33" t="inlineStr">
         <is>
@@ -17495,9 +17781,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B81" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B81" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C81" s="33" t="inlineStr">
         <is>
@@ -17789,9 +18076,10 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B85" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B85" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C85" s="33" t="inlineStr">
         <is>
@@ -17874,9 +18162,10 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B86" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B86" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C86" s="33" t="inlineStr">
         <is>
@@ -17959,9 +18248,10 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B87" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B87" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C87" s="33" t="inlineStr">
         <is>
@@ -18044,9 +18334,10 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B88" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
-        <v/>
+      <c r="B88" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
+        </is>
       </c>
       <c r="C88" s="33" t="inlineStr">
         <is>
@@ -18129,9 +18420,10 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B89" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B89" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C89" s="33" t="inlineStr">
         <is>
@@ -18214,9 +18506,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B90" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B90" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C90" s="33" t="inlineStr">
         <is>
@@ -18497,9 +18790,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B94" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B94" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C94" s="33" t="inlineStr">
         <is>
@@ -18582,9 +18876,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B95" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B95" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C95" s="33" t="inlineStr">
         <is>
@@ -18667,9 +18962,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B96" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B96" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C96" s="33" t="inlineStr">
         <is>
@@ -18752,9 +19048,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B97" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B97" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C97" s="33" t="inlineStr">
         <is>
@@ -18837,9 +19134,10 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B98" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
-        <v/>
+      <c r="B98" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C98" s="33" t="inlineStr">
         <is>
@@ -18922,9 +19220,10 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B99" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
-        <v/>
+      <c r="B99" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C99" s="33" t="inlineStr">
         <is>
@@ -19007,9 +19306,10 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B100" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
-        <v/>
+      <c r="B100" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C100" s="33" t="inlineStr">
         <is>
@@ -19092,9 +19392,10 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B101" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
-        <v/>
+      <c r="B101" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C101" s="33" t="inlineStr">
         <is>
@@ -19177,9 +19478,10 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B102" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
-        <v/>
+      <c r="B102" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C102" s="33" t="inlineStr">
         <is>
@@ -19262,9 +19564,10 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B103" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
-        <v/>
+      <c r="B103" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
+        </is>
       </c>
       <c r="C103" s="33" t="inlineStr">
         <is>
@@ -19347,9 +19650,10 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B104" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
-        <v/>
+      <c r="B104" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C104" s="33" t="inlineStr">
         <is>
@@ -19432,9 +19736,10 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B105" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
-        <v/>
+      <c r="B105" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C105" s="33" t="inlineStr">
         <is>
@@ -19517,9 +19822,10 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B106" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
-        <v/>
+      <c r="B106" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
+        </is>
       </c>
       <c r="C106" s="33" t="inlineStr">
         <is>
@@ -19800,9 +20106,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B110" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B110" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C110" s="33" t="inlineStr">
         <is>
@@ -19885,9 +20192,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B111" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B111" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C111" s="33" t="inlineStr">
         <is>
@@ -19970,9 +20278,10 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B112" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
-        <v/>
+      <c r="B112" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+        </is>
       </c>
       <c r="C112" s="33" t="inlineStr">
         <is>
@@ -20055,9 +20364,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B113" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B113" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C113" s="33" t="inlineStr">
         <is>
@@ -20140,9 +20450,10 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B114" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
-        <v/>
+      <c r="B114" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+        </is>
       </c>
       <c r="C114" s="33" t="inlineStr">
         <is>
@@ -20225,9 +20536,10 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B115" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
+      <c r="B115" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
       </c>
       <c r="C115" s="33" t="inlineStr">
         <is>
@@ -20310,9 +20622,10 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B116" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
-        <v/>
+      <c r="B116" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C116" s="33" t="inlineStr">
         <is>
@@ -20395,9 +20708,10 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B117" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
-        <v/>
+      <c r="B117" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C117" s="33" t="inlineStr">
         <is>
@@ -20480,9 +20794,10 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B118" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
-        <v/>
+      <c r="B118" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+        </is>
       </c>
       <c r="C118" s="33" t="inlineStr">
         <is>
@@ -20565,9 +20880,10 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B119" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
-        <v/>
+      <c r="B119" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+        </is>
       </c>
       <c r="C119" s="33" t="inlineStr">
         <is>
@@ -20650,9 +20966,10 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B120" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
-        <v/>
+      <c r="B120" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+        </is>
       </c>
       <c r="C120" s="33" t="inlineStr">
         <is>
@@ -20735,9 +21052,10 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B121" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
-        <v/>
+      <c r="B121" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
       </c>
       <c r="C121" s="33" t="inlineStr">
         <is>
@@ -20877,9 +21195,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B125" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B125" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C125" s="33" t="inlineStr">
         <is>
@@ -20918,9 +21237,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B126" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B126" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C126" s="33" t="inlineStr">
         <is>
@@ -20978,56 +21298,124 @@
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing-1'!B2" tooltip="Back to column B on Application Attribute Testing-1" display="1. Application Name (column B): review of evidence files and results"/>
     <hyperlink ref="A5" location="'Testing Attributes Testing -2'!A110" tooltip="Go to MA01 evidence review" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId1"/>
     <hyperlink ref="A7" location="'Application Attribute Testing-1'!C2" tooltip="Back to column C on Application Attribute Testing-1" display="2. Applications in Scope Identified (column C): review of evidence files and results"/>
     <hyperlink ref="A9" location="'Testing Attributes Testing -2'!A110" tooltip="Go to MA01 evidence review" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId2"/>
     <hyperlink ref="A10" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId3"/>
     <hyperlink ref="A11" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId4"/>
     <hyperlink ref="A13" location="'Application Attribute Testing-1'!D2" tooltip="Back to column D on Application Attribute Testing-1" display="3. IT DR exercise name (column D): review of evidence files and results"/>
     <hyperlink ref="A15" location="'Testing Attributes Testing -2'!A111" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId5"/>
     <hyperlink ref="A16" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId6"/>
     <hyperlink ref="A17" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId7"/>
     <hyperlink ref="A19" location="'Application Attribute Testing-1'!E2" tooltip="Back to column E on Application Attribute Testing-1" display="4. IT DR exercise name, was the exercise annually executed? (column E): review of evidence files and results"/>
     <hyperlink ref="A21" location="'Testing Attributes Testing -2'!A111" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId8"/>
     <hyperlink ref="A22" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId9"/>
     <hyperlink ref="A23" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId10"/>
     <hyperlink ref="A25" location="'Application Attribute Testing-1'!F2" tooltip="Back to column F on Application Attribute Testing-1" display="5. Business Tester (column F): review of evidence files and results"/>
     <hyperlink ref="A27" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId11"/>
     <hyperlink ref="A29" location="'Application Attribute Testing-1'!G2" tooltip="Back to column G on Application Attribute Testing-1" display="6. Business Data validation (column G): review of evidence files and results"/>
     <hyperlink ref="A31" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId12"/>
     <hyperlink ref="A33" location="'Application Attribute Testing-1'!H2" tooltip="Back to column H on Application Attribute Testing-1" display="7. Business line manager name (column H): review of evidence files and results"/>
     <hyperlink ref="A35" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId13"/>
     <hyperlink ref="A36" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId14"/>
     <hyperlink ref="A38" location="'Application Attribute Testing-1'!I2" tooltip="Back to column I on Application Attribute Testing-1" display="8. Business line manager approval dates (column I): review of evidence files and results"/>
     <hyperlink ref="A40" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId15"/>
     <hyperlink ref="A42" location="'Application Attribute Testing-1'!J2" tooltip="Back to column J on Application Attribute Testing-1" display="9. DIV Test procedures listed within the Test results document (column J): review of evidence files and results"/>
     <hyperlink ref="A44" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId16"/>
     <hyperlink ref="A46" location="'Application Attribute Testing-1'!K2" tooltip="Back to column K on Application Attribute Testing-1" display="10. Emails showing Business line manager approval of DIV testing results (column K): review of evidence files and results"/>
     <hyperlink ref="A48" location="'Testing Attributes Testing -2'!A90" tooltip="Go to BLA06 evidence review" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId17"/>
     <hyperlink ref="A49" location="'Testing Attributes Testing -2'!A94" tooltip="Go to DMA01 evidence review" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId18"/>
     <hyperlink ref="A50" location="'Testing Attributes Testing -2'!A95" tooltip="Go to DMA02 evidence review" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId19"/>
     <hyperlink ref="A51" location="'Testing Attributes Testing -2'!A96" tooltip="Go to DMA03 evidence review" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId20"/>
     <hyperlink ref="A52" location="'Testing Attributes Testing -2'!A97" tooltip="Go to DMA04 evidence review" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId21"/>
     <hyperlink ref="A54" location="'Application Attribute Testing-1'!L2" tooltip="Back to column L on Application Attribute Testing-1" display="11. All evidence of Data Integrity DR test in BCIC (column L): review of evidence files and results"/>
     <hyperlink ref="A56" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId22"/>
     <hyperlink ref="A58" location="'Application Attribute Testing-1'!M2" tooltip="Back to column M on Application Attribute Testing-1" display="12. Annual Testing Executed (column M): review of evidence files and results"/>
     <hyperlink ref="A60" location="'Testing Attributes Testing -2'!A111" tooltip="Go to E01 evidence review" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId23"/>
     <hyperlink ref="A61" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId24"/>
     <hyperlink ref="A62" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId25"/>
     <hyperlink ref="A64" location="'Application Attribute Testing-1'!N2" tooltip="Back to column N on Application Attribute Testing-1" display="13. Data Integrity Validation Performed by IT DR Team (column N): review of evidence files and results"/>
     <hyperlink ref="A66" location="'Testing Attributes Testing -2'!A115" tooltip="Go to E05 evidence review" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId26"/>
     <hyperlink ref="A67" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId27"/>
     <hyperlink ref="A68" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId28"/>
     <hyperlink ref="A70" location="'Application Attribute Testing-1'!O2" tooltip="Back to column O on Application Attribute Testing-1" display="14. Business Line Approval of Results (column O): review of evidence files and results"/>
     <hyperlink ref="A72" location="'Testing Attributes Testing -2'!A90" tooltip="Go to BLA06 evidence review" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId29"/>
     <hyperlink ref="A73" location="'Testing Attributes Testing -2'!A94" tooltip="Go to DMA01 evidence review" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId30"/>
     <hyperlink ref="A74" location="'Testing Attributes Testing -2'!A95" tooltip="Go to DMA02 evidence review" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId31"/>
     <hyperlink ref="A75" location="'Testing Attributes Testing -2'!A96" tooltip="Go to DMA03 evidence review" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId32"/>
     <hyperlink ref="A76" location="'Testing Attributes Testing -2'!A97" tooltip="Go to DMA04 evidence review" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId33"/>
     <hyperlink ref="A77" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId34"/>
     <hyperlink ref="A79" location="'Application Attribute Testing-1'!P2" tooltip="Back to column P on Application Attribute Testing-1" display="15. Results Documented in BCMS (column P): review of evidence files and results"/>
     <hyperlink ref="A81" location="'Testing Attributes Testing -2'!A113" tooltip="Go to E03 evidence review" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B121" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx" r:id="rId66"/>
     <hyperlink ref="A125" location="'Application Attribute Testing-1'!R3" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId67"/>
     <hyperlink ref="A126" location="'Application Attribute Testing-1'!R3" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -22473,9 +22861,10 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B3" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B3" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C3" s="33" t="inlineStr">
         <is>
@@ -22564,9 +22953,10 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B4" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B4" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C4" s="33" t="inlineStr">
         <is>
@@ -22655,9 +23045,10 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B5" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
         <is>
@@ -22746,9 +23137,10 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B6" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
-        <v/>
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
+        </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
         <is>
@@ -22837,9 +23229,10 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B7" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
+      <c r="B7" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
+        </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
@@ -22928,9 +23321,10 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B8" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
+      <c r="B8" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
       </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
@@ -23016,9 +23410,10 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B9" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
+      <c r="B9" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
@@ -23104,9 +23499,10 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B10" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
+      <c r="B10" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
@@ -23197,9 +23593,10 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B11" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
+      <c r="B11" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
@@ -23285,9 +23682,10 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B12" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
+      <c r="B12" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
       </c>
       <c r="C12" s="33" t="inlineStr">
         <is>
@@ -23373,9 +23771,10 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B13" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
-        <v/>
+      <c r="B13" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
+        </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
@@ -23461,9 +23860,10 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B14" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
-        <v/>
+      <c r="B14" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
@@ -23549,9 +23949,10 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B15" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
-        <v/>
+      <c r="B15" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
@@ -23637,9 +24038,10 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B16" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
-        <v/>
+      <c r="B16" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
@@ -23725,9 +24127,10 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B17" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
-        <v/>
+      <c r="B17" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
+        </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
@@ -23813,9 +24216,10 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B18" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
-        <v/>
+      <c r="B18" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
+        </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
@@ -23901,9 +24305,10 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B19" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
-        <v/>
+      <c r="B19" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
@@ -23989,9 +24394,10 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B20" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
-        <v/>
+      <c r="B20" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
+        </is>
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
@@ -24077,9 +24483,10 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B21" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
-        <v/>
+      <c r="B21" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
+        </is>
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
@@ -24158,9 +24565,10 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B22" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
+      <c r="B22" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -24245,9 +24653,10 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B23" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
+      <c r="B23" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
       </c>
       <c r="C23" s="33" t="inlineStr">
         <is>
@@ -24335,9 +24744,10 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B24" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
-        <v/>
+      <c r="B24" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+        </is>
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
@@ -24422,9 +24832,10 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B25" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
+      <c r="B25" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
@@ -24518,9 +24929,10 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B26" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
-        <v/>
+      <c r="B26" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+        </is>
       </c>
       <c r="C26" s="33" t="inlineStr">
         <is>
@@ -24608,9 +25020,10 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B27" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
+      <c r="B27" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
@@ -24694,9 +25107,10 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B28" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
-        <v/>
+      <c r="B28" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
@@ -24779,9 +25193,10 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B29" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
-        <v/>
+      <c r="B29" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+        </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
@@ -24865,9 +25280,10 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B30" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
-        <v/>
+      <c r="B30" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+        </is>
       </c>
       <c r="C30" s="33" t="inlineStr">
         <is>
@@ -24956,9 +25372,10 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B31" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
-        <v/>
+      <c r="B31" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+        </is>
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
@@ -25041,9 +25458,10 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B32" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
-        <v/>
+      <c r="B32" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+        </is>
       </c>
       <c r="C32" s="33" t="inlineStr">
         <is>
@@ -25122,9 +25540,10 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B33" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
-        <v/>
+      <c r="B33" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
@@ -25212,9 +25631,10 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B34" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B34" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
@@ -25258,9 +25678,10 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B35" s="24">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
+      <c r="B35" s="83" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
@@ -25306,38 +25727,71 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing'!A73" display="BLA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf" r:id="rId1"/>
     <hyperlink ref="A4" location="'Application Attribute Testing'!A74" display="BLA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf" r:id="rId2"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A75" display="BLA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf" r:id="rId3"/>
     <hyperlink ref="A6" location="'Application Attribute Testing'!A76" display="BLA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx" r:id="rId4"/>
     <hyperlink ref="A7" location="'Application Attribute Testing'!A77" display="BLA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf" r:id="rId5"/>
     <hyperlink ref="A8" location="'Application Attribute Testing'!A78" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId6"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A82" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId7"/>
     <hyperlink ref="A10" location="'Application Attribute Testing'!A83" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId8"/>
     <hyperlink ref="A11" location="'Application Attribute Testing'!A84" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId9"/>
     <hyperlink ref="A12" location="'Application Attribute Testing'!A85" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId10"/>
     <hyperlink ref="A13" location="'Application Attribute Testing'!A86" display="DMA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg" r:id="rId11"/>
     <hyperlink ref="A14" location="'Application Attribute Testing'!A87" display="DMA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg" r:id="rId12"/>
     <hyperlink ref="A15" location="'Application Attribute Testing'!A88" display="DMA07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg" r:id="rId13"/>
     <hyperlink ref="A16" location="'Application Attribute Testing'!A89" display="DMA08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg" r:id="rId14"/>
     <hyperlink ref="A17" location="'Application Attribute Testing'!A90" display="DMA09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg" r:id="rId15"/>
     <hyperlink ref="A18" location="'Application Attribute Testing'!A91" display="DMA10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml" r:id="rId16"/>
     <hyperlink ref="A19" location="'Application Attribute Testing'!A92" display="DMA11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml" r:id="rId17"/>
     <hyperlink ref="A20" location="'Application Attribute Testing'!A93" display="DMA12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml" r:id="rId18"/>
     <hyperlink ref="A21" location="'Application Attribute Testing'!A94" display="DMA13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml" r:id="rId19"/>
     <hyperlink ref="A22" location="'Application Attribute Testing'!A98" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png" r:id="rId20"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A99" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId21"/>
     <hyperlink ref="A24" location="'Application Attribute Testing'!A100" display="E02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg" r:id="rId22"/>
     <hyperlink ref="A25" location="'Application Attribute Testing'!A101" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId23"/>
     <hyperlink ref="A26" location="'Application Attribute Testing'!A102" display="E04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg" r:id="rId24"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A103" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId25"/>
     <hyperlink ref="A28" location="'Application Attribute Testing'!A104" display="E07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg" r:id="rId26"/>
     <hyperlink ref="A29" location="'Application Attribute Testing'!A105" display="E08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg" r:id="rId27"/>
     <hyperlink ref="A30" location="'Application Attribute Testing'!A106" display="E09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg" r:id="rId28"/>
     <hyperlink ref="A31" location="'Application Attribute Testing'!A107" display="E10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg" r:id="rId29"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A108" display="E13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg" r:id="rId30"/>
     <hyperlink ref="A33" location="'Application Attribute Testing'!A109" display="E16b"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx" r:id="rId31"/>
     <hyperlink ref="A34" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId32"/>
     <hyperlink ref="A35" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -25405,6 +25859,7 @@
       <c r="P2" s="70" t="n"/>
       <c r="Q2" s="70" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="51" t="inlineStr">
         <is>
@@ -27199,6 +27654,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15.6" customHeight="1">
       <c r="A16" s="53" t="inlineStr">
         <is>
@@ -27400,13 +27856,15 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B3" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"MA01_BSI In-Scope Applications-2026.png")</f>
-        <v/>
-      </c>
-      <c r="C3" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications")</f>
-        <v/>
+      <c r="B3" s="84" t="inlineStr">
+        <is>
+          <t>MA01_BSI In-Scope Applications-2026.png</t>
+        </is>
+      </c>
+      <c r="C3" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications</t>
+        </is>
       </c>
       <c r="D3" s="57" t="inlineStr">
         <is>
@@ -27452,13 +27910,15 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B4" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
-      </c>
-      <c r="C4" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B4" s="84" t="inlineStr">
+        <is>
+          <t>BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
+        </is>
+      </c>
+      <c r="C4" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D4" s="57" t="inlineStr">
         <is>
@@ -27504,13 +27964,15 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B5" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
-      </c>
-      <c r="C5" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B5" s="84" t="inlineStr">
+        <is>
+          <t>BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
+        </is>
+      </c>
+      <c r="C5" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D5" s="57" t="inlineStr">
         <is>
@@ -27556,13 +28018,15 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B6" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
-      </c>
-      <c r="C6" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B6" s="84" t="inlineStr">
+        <is>
+          <t>BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
+        </is>
+      </c>
+      <c r="C6" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D6" s="57" t="inlineStr">
         <is>
@@ -27608,13 +28072,15 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B7" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
-        <v/>
-      </c>
-      <c r="C7" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B7" s="84" t="inlineStr">
+        <is>
+          <t>BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
+        </is>
+      </c>
+      <c r="C7" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D7" s="57" t="inlineStr">
         <is>
@@ -27660,13 +28126,15 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B8" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
-        <v/>
-      </c>
-      <c r="C8" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B8" s="84" t="inlineStr">
+        <is>
+          <t>BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
+        </is>
+      </c>
+      <c r="C8" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D8" s="57" t="inlineStr">
         <is>
@@ -27712,13 +28180,15 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B9" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C9" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
-        <v/>
+      <c r="B9" s="84" t="inlineStr">
+        <is>
+          <t>BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+        </is>
+      </c>
+      <c r="C9" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+        </is>
       </c>
       <c r="D9" s="57" t="inlineStr">
         <is>
@@ -27764,13 +28234,15 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B10" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C10" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B10" s="84" t="inlineStr">
+        <is>
+          <t>DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C10" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D10" s="57" t="inlineStr">
         <is>
@@ -27816,13 +28288,15 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B11" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C11" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B11" s="84" t="inlineStr">
+        <is>
+          <t>DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+        </is>
+      </c>
+      <c r="C11" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D11" s="57" t="inlineStr">
         <is>
@@ -27868,13 +28342,15 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B12" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C12" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B12" s="84" t="inlineStr">
+        <is>
+          <t>DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C12" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D12" s="57" t="inlineStr">
         <is>
@@ -27920,13 +28396,15 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B13" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C13" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+        </is>
+      </c>
+      <c r="C13" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D13" s="57" t="inlineStr">
         <is>
@@ -27972,13 +28450,15 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B14" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C14" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B14" s="84" t="inlineStr">
+        <is>
+          <t>DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
+        </is>
+      </c>
+      <c r="C14" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D14" s="57" t="inlineStr">
         <is>
@@ -28024,13 +28504,15 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B15" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C15" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B15" s="84" t="inlineStr">
+        <is>
+          <t>DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C15" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D15" s="57" t="inlineStr">
         <is>
@@ -28076,13 +28558,15 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B16" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C16" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C16" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D16" s="57" t="inlineStr">
         <is>
@@ -28128,13 +28612,15 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B17" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C17" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C17" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D17" s="57" t="inlineStr">
         <is>
@@ -28180,13 +28666,15 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B18" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
-        <v/>
-      </c>
-      <c r="C18" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B18" s="84" t="inlineStr">
+        <is>
+          <t>DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
+        </is>
+      </c>
+      <c r="C18" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D18" s="57" t="inlineStr">
         <is>
@@ -28232,13 +28720,15 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B19" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
-        <v/>
-      </c>
-      <c r="C19" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B19" s="84" t="inlineStr">
+        <is>
+          <t>DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
+        </is>
+      </c>
+      <c r="C19" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D19" s="57" t="inlineStr">
         <is>
@@ -28284,13 +28774,15 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B20" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
-        <v/>
-      </c>
-      <c r="C20" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B20" s="84" t="inlineStr">
+        <is>
+          <t>DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
+        </is>
+      </c>
+      <c r="C20" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D20" s="57" t="inlineStr">
         <is>
@@ -28336,13 +28828,15 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B21" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
-        <v/>
-      </c>
-      <c r="C21" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B21" s="84" t="inlineStr">
+        <is>
+          <t>DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
+        </is>
+      </c>
+      <c r="C21" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D21" s="57" t="inlineStr">
         <is>
@@ -28388,13 +28882,15 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B22" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
-        <v/>
-      </c>
-      <c r="C22" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
-        <v/>
+      <c r="B22" s="84" t="inlineStr">
+        <is>
+          <t>DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
+        </is>
+      </c>
+      <c r="C22" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+        </is>
       </c>
       <c r="D22" s="57" t="inlineStr">
         <is>
@@ -28436,13 +28932,15 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B23" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
-        <v/>
-      </c>
-      <c r="C23" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B23" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+        </is>
+      </c>
+      <c r="C23" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D23" s="57" t="inlineStr">
         <is>
@@ -28488,13 +28986,15 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B24" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
-        <v/>
-      </c>
-      <c r="C24" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B24" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+        </is>
+      </c>
+      <c r="C24" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D24" s="57" t="inlineStr">
         <is>
@@ -28540,13 +29040,15 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B25" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
-        <v/>
-      </c>
-      <c r="C25" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B25" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+        </is>
+      </c>
+      <c r="C25" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D25" s="57" t="inlineStr">
         <is>
@@ -28592,13 +29094,15 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B26" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
-        <v/>
-      </c>
-      <c r="C26" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B26" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+        </is>
+      </c>
+      <c r="C26" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D26" s="57" t="inlineStr">
         <is>
@@ -28644,13 +29148,15 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B27" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
-        <v/>
-      </c>
-      <c r="C27" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B27" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+        </is>
+      </c>
+      <c r="C27" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D27" s="57" t="inlineStr">
         <is>
@@ -28696,13 +29202,15 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B28" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
-        <v/>
-      </c>
-      <c r="C28" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B28" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+        </is>
+      </c>
+      <c r="C28" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D28" s="57" t="inlineStr">
         <is>
@@ -28748,13 +29256,15 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B29" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
-        <v/>
-      </c>
-      <c r="C29" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B29" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+        </is>
+      </c>
+      <c r="C29" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D29" s="57" t="inlineStr">
         <is>
@@ -28800,13 +29310,15 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B30" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
-        <v/>
-      </c>
-      <c r="C30" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B30" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+        </is>
+      </c>
+      <c r="C30" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D30" s="57" t="inlineStr">
         <is>
@@ -28852,13 +29364,15 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B31" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
-        <v/>
-      </c>
-      <c r="C31" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B31" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+        </is>
+      </c>
+      <c r="C31" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D31" s="57" t="inlineStr">
         <is>
@@ -28904,13 +29418,15 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B32" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
-        <v/>
-      </c>
-      <c r="C32" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B32" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+        </is>
+      </c>
+      <c r="C32" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D32" s="57" t="inlineStr">
         <is>
@@ -28952,13 +29468,15 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B33" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
-        <v/>
-      </c>
-      <c r="C33" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
-        <v/>
+      <c r="B33" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
+      </c>
+      <c r="C33" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
       </c>
       <c r="D33" s="57" t="inlineStr">
         <is>
@@ -29004,13 +29522,15 @@
           <t>DRS01</t>
         </is>
       </c>
-      <c r="B34" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml")</f>
-        <v/>
-      </c>
-      <c r="C34" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails")</f>
-        <v/>
+      <c r="B34" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml</t>
+        </is>
+      </c>
+      <c r="C34" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails</t>
+        </is>
       </c>
       <c r="D34" s="57" t="inlineStr">
         <is>
@@ -29059,13 +29579,15 @@
           <t>DRS02</t>
         </is>
       </c>
-      <c r="B35" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml")</f>
-        <v/>
-      </c>
-      <c r="C35" s="56">
-        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("05_Annual_DR_Exercise_IT_and_Business_Scope_Emails","\","/"),"05_Annual_DR_Exercise_IT_and_Business_Scope_Emails"),"BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails")</f>
-        <v/>
+      <c r="B35" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml</t>
+        </is>
+      </c>
+      <c r="C35" s="84" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails</t>
+        </is>
       </c>
       <c r="D35" s="57" t="inlineStr">
         <is>
@@ -30814,38 +31336,104 @@
   <autoFilter ref="A2:K35"/>
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing'!A98" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" display="MA01_BSI In-Scope Applications-2026.png" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" display="BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications" r:id="rId2"/>
     <hyperlink ref="A4" location="'Application Attribute Testing'!A73" display="BLA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" display="BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId4"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A74" display="BLA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId6"/>
     <hyperlink ref="A6" location="'Application Attribute Testing'!A75" display="BLA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" display="BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId8"/>
     <hyperlink ref="A7" location="'Application Attribute Testing'!A76" display="BLA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" display="BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId10"/>
     <hyperlink ref="A8" location="'Application Attribute Testing'!A77" display="BLA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" display="BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId12"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A78" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" display="BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" display="BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email" r:id="rId14"/>
     <hyperlink ref="A10" location="'Application Attribute Testing'!A82" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" display="DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId16"/>
     <hyperlink ref="A11" location="'Application Attribute Testing'!A83" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" display="DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId18"/>
     <hyperlink ref="A12" location="'Application Attribute Testing'!A84" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" display="DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId20"/>
     <hyperlink ref="A13" location="'Application Attribute Testing'!A85" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" display="DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId22"/>
     <hyperlink ref="A14" location="'Application Attribute Testing'!A86" display="DMA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" display="DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId24"/>
     <hyperlink ref="A15" location="'Application Attribute Testing'!A87" display="DMA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" display="DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId26"/>
     <hyperlink ref="A16" location="'Application Attribute Testing'!A88" display="DMA07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" display="DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId28"/>
     <hyperlink ref="A17" location="'Application Attribute Testing'!A89" display="DMA08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" display="DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId30"/>
     <hyperlink ref="A18" location="'Application Attribute Testing'!A90" display="DMA09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" display="DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId32"/>
     <hyperlink ref="A19" location="'Application Attribute Testing'!A91" display="DMA10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" display="DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId34"/>
     <hyperlink ref="A20" location="'Application Attribute Testing'!A92" display="DMA11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" display="DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId36"/>
     <hyperlink ref="A21" location="'Application Attribute Testing'!A93" display="DMA12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId38"/>
     <hyperlink ref="A22" location="'Application Attribute Testing'!A94" display="DMA13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" display="DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" display="BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals" r:id="rId40"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A99" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" display="BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId42"/>
     <hyperlink ref="A24" location="'Application Attribute Testing'!A100" display="E02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" display="BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId44"/>
     <hyperlink ref="A25" location="'Application Attribute Testing'!A101" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" display="BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId46"/>
     <hyperlink ref="A26" location="'Application Attribute Testing'!A102" display="E04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" display="BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId48"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A103" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" display="BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId50"/>
     <hyperlink ref="A28" location="'Application Attribute Testing'!A104" display="E07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" display="BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId52"/>
     <hyperlink ref="A29" location="'Application Attribute Testing'!A105" display="E08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" display="BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId54"/>
     <hyperlink ref="A30" location="'Application Attribute Testing'!A106" display="E09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" display="BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId56"/>
     <hyperlink ref="A31" location="'Application Attribute Testing'!A107" display="E10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" display="BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId58"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A108" display="E13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" display="BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId60"/>
     <hyperlink ref="A33" location="'Application Attribute Testing'!A109" display="E16b"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" display="BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" display="BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence" r:id="rId62"/>
     <hyperlink ref="A34" location="'Testing Attributes Testing -2'!A125" display="DRS01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS01_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - IT Scope 10-08-2025.eml" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails" r:id="rId64"/>
     <hyperlink ref="A35" location="'Testing Attributes Testing -2'!A126" display="DRS02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails\DRS02_Fw_ Annual DR (Disaster Recovery) Exercise - Saturday, Nov 15 - confirm participants - Business Scope 10-08-2025.eml" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" display="BSI.IT.6.C7.3-Evidences\05_Annual_DR_Exercise_IT_and_Business_Scope_Emails" r:id="rId66"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>